<commit_message>
some analyze and graph scripts
</commit_message>
<xml_diff>
--- a/statistick/my_eval_2.xlsx
+++ b/statistick/my_eval_2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RAG-eval\DP-evaluation\statistick\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE141BAD-AF02-4370-B9B7-D8ED652FE2A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9306FA43-CA71-4FE0-856A-ADEE696EE1FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5520" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Slepý Test SET 2" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="132">
   <si>
     <t>Otázka</t>
   </si>
@@ -1724,12 +1724,24 @@
       <c r="C15" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
+      <c r="D15" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>119</v>
+      </c>
       <c r="J15" s="1" t="s">
         <v>99</v>
       </c>

</xml_diff>